<commit_message>
feat: add role-based recruiting and OCR workflows
</commit_message>
<xml_diff>
--- a/docs/TalentHub_專案時程表.xlsx
+++ b/docs/TalentHub_專案時程表.xlsx
@@ -1,17 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="甘特圖" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="里程碑一覽" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="階段任務明細" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="本次工作流進度" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="甘特圖" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="里程碑一覽" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="階段任務明細" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'本次工作流進度'!$A$2:$D$6</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -19,7 +22,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="10">
+  <fonts count="12">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -66,8 +69,17 @@
       <color rgb="00C00000"/>
       <sz val="9"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="15"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="0017324D"/>
+    </font>
   </fonts>
-  <fills count="15">
+  <fills count="19">
     <fill>
       <patternFill/>
     </fill>
@@ -152,8 +164,28 @@
         <bgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0017324D"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="000E7490"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EAF5F7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFFFF"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -175,11 +207,93 @@
         <color rgb="00D9D9D9"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00D9D9D9"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00D9D9D9"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D9D9D9"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00D9D9D9"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D9D9D9"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00D9D9D9"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D9D9D9"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D9D9D9"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00D9D9D9"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00D9D9D9"/>
+      </left>
+      <right style="thin">
+        <color rgb="00D9D9D9"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00D9D9D9"/>
+      </left>
+      <right style="thin">
+        <color rgb="00D9D9D9"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00D9D9D9"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <bottom style="thin">
+        <color rgb="00D9E2EC"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="47">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -274,6 +388,27 @@
     <xf numFmtId="0" fontId="0" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="15" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="16" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="18" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -637,6 +772,162 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="29" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="43" customWidth="1" min="3" max="3"/>
+    <col width="38" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="38" t="inlineStr">
+        <is>
+          <t>TalentHub 本次平行工作流進度（2026-07-14）</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="39" t="inlineStr">
+        <is>
+          <t>工作流</t>
+        </is>
+      </c>
+      <c r="B2" s="39" t="inlineStr">
+        <is>
+          <t>狀態</t>
+        </is>
+      </c>
+      <c r="C2" s="39" t="inlineStr">
+        <is>
+          <t>本次交付</t>
+        </is>
+      </c>
+      <c r="D2" s="39" t="inlineStr">
+        <is>
+          <t>正式上線前下一關</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="38" customHeight="1">
+      <c r="A3" s="40" t="inlineStr">
+        <is>
+          <t>多角色權限與資料範圍</t>
+        </is>
+      </c>
+      <c r="B3" s="40" t="inlineStr">
+        <is>
+          <t>已完成 MVP</t>
+        </is>
+      </c>
+      <c r="C3" s="40" t="inlineStr">
+        <is>
+          <t>IT／HR／主管依角色與資料範圍操作</t>
+        </is>
+      </c>
+      <c r="D3" s="40" t="inlineStr">
+        <is>
+          <t>三角色 UAT 與越權測試</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="38" customHeight="1">
+      <c r="A4" s="41" t="inlineStr">
+        <is>
+          <t>104／1111 OCR 固定欄位入庫</t>
+        </is>
+      </c>
+      <c r="B4" s="41" t="inlineStr">
+        <is>
+          <t>已完成 MVP</t>
+        </is>
+      </c>
+      <c r="C4" s="41" t="inlineStr">
+        <is>
+          <t>來源模板、固定欄位、信心分數、校對後入庫</t>
+        </is>
+      </c>
+      <c r="D4" s="41" t="inlineStr">
+        <is>
+          <t>各 10 份授權去識別樣本校準</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="38" customHeight="1">
+      <c r="A5" s="40" t="inlineStr">
+        <is>
+          <t>可解釋人才職缺配對</t>
+        </is>
+      </c>
+      <c r="B5" s="40" t="inlineStr">
+        <is>
+          <t>已完成 MVP</t>
+        </is>
+      </c>
+      <c r="C5" s="40" t="inlineStr">
+        <is>
+          <t>必要條件與多面向分數、排序原因</t>
+        </is>
+      </c>
+      <c r="D5" s="40" t="inlineStr">
+        <is>
+          <t>HR 校準權重與公平性檢核</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="38" customHeight="1">
+      <c r="A6" s="41" t="inlineStr">
+        <is>
+          <t>角色化互動介面／官網整合</t>
+        </is>
+      </c>
+      <c r="B6" s="41" t="inlineStr">
+        <is>
+          <t>已完成介面基線</t>
+        </is>
+      </c>
+      <c r="C6" s="41" t="inlineStr">
+        <is>
+          <t>角色導覽、任務提示、響應式工作台</t>
+        </is>
+      </c>
+      <c r="D6" s="41" t="inlineStr">
+        <is>
+          <t>公司 Logo／色票／導覽／SSO 規格</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="42" t="inlineStr">
+        <is>
+          <t>說明</t>
+        </is>
+      </c>
+      <c r="B8" s="43" t="inlineStr">
+        <is>
+          <t>「已完成 MVP」供內部展示／試用；正式處理真實個資前仍需樣本校準、資安檢核與 UAT。</t>
+        </is>
+      </c>
+      <c r="C8" s="43" t="n"/>
+      <c r="D8" s="43" t="n"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A2:D6"/>
+  <mergeCells count="2">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="B8:D8"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:Z13"/>
@@ -680,7 +971,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>啟動 2026-07-20 ｜ 方案A：1 名全端工程師（詳 docs/07）｜ 產生日 2026-07-13 ｜ 色塊＝工作期間，◆＝里程碑</t>
+          <t>啟動 2026-07-20 ｜ v1.2：2026-07-14 更新 ｜ 色塊＝工作期間，◆＝里程碑</t>
         </is>
       </c>
     </row>
@@ -715,28 +1006,49 @@
           <t>7月</t>
         </is>
       </c>
+      <c r="G3" s="44" t="n"/>
+      <c r="H3" s="45" t="n"/>
       <c r="I3" s="4" t="inlineStr">
         <is>
           <t>8月</t>
         </is>
       </c>
+      <c r="J3" s="44" t="n"/>
+      <c r="K3" s="44" t="n"/>
+      <c r="L3" s="44" t="n"/>
+      <c r="M3" s="45" t="n"/>
       <c r="N3" s="4" t="inlineStr">
         <is>
           <t>9月</t>
         </is>
       </c>
+      <c r="O3" s="44" t="n"/>
+      <c r="P3" s="44" t="n"/>
+      <c r="Q3" s="45" t="n"/>
       <c r="R3" s="4" t="inlineStr">
         <is>
           <t>10月</t>
         </is>
       </c>
+      <c r="S3" s="44" t="n"/>
+      <c r="T3" s="44" t="n"/>
+      <c r="U3" s="45" t="n"/>
       <c r="V3" s="4" t="inlineStr">
         <is>
           <t>11月</t>
         </is>
       </c>
+      <c r="W3" s="44" t="n"/>
+      <c r="X3" s="44" t="n"/>
+      <c r="Y3" s="44" t="n"/>
+      <c r="Z3" s="45" t="n"/>
     </row>
     <row r="4">
+      <c r="A4" s="46" t="n"/>
+      <c r="B4" s="46" t="n"/>
+      <c r="C4" s="46" t="n"/>
+      <c r="D4" s="46" t="n"/>
+      <c r="E4" s="46" t="n"/>
       <c r="F4" s="5" t="inlineStr">
         <is>
           <t>7/13</t>
@@ -1335,7 +1647,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1509,7 +1821,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
feat: matching evaluation report; sync docs & timeline to current progress
- add GET /reports/matching-evaluation (precision@K, recall@K, gate
  false-negatives, score calibration, rank effectiveness) with tests
- update docs to reflect the matching accuracy work, auth/upload/deploy
  hardening, new endpoints/columns, and current milestone completion status
  (docs 02, 05, 07, 08, 10, 11 + the project schedule .xlsx)
- remove the two static diagram HTML exports under docs/

Validated: 109 backend tests pass, ruff clean.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/TalentHub_專案時程表.xlsx
+++ b/docs/TalentHub_專案時程表.xlsx
@@ -774,19 +774,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
     <col width="43" customWidth="1" min="3" max="3"/>
     <col width="38" customWidth="1" min="4" max="4"/>
+    <col width="54" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="38" t="inlineStr">
         <is>
-          <t>TalentHub 本次平行工作流進度（2026-07-14）</t>
+          <t>TalentHub 平行工作流進度（更新至 2026-07-16）</t>
         </is>
       </c>
     </row>
@@ -811,6 +812,11 @@
           <t>正式上線前下一關</t>
         </is>
       </c>
+      <c r="E2" s="39" t="inlineStr">
+        <is>
+          <t>現況（2026-07-16）</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="38" customHeight="1">
       <c r="A3" s="40" t="inlineStr">
@@ -833,6 +839,11 @@
           <t>三角色 UAT 與越權測試</t>
         </is>
       </c>
+      <c r="E3" s="40" t="inlineStr">
+        <is>
+          <t>已上線；認證強化：帳號級自動過期鎖定、強制首登改密、密碼重設令 token 失效、refresh 重用偵測</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="38" customHeight="1">
       <c r="A4" s="41" t="inlineStr">
@@ -855,6 +866,11 @@
           <t>各 10 份授權去識別樣本校準</t>
         </is>
       </c>
+      <c r="E4" s="41" t="inlineStr">
+        <is>
+          <t>解析／OCR／去重／並排校對已上線；上傳安全：非 dev fail-closed 掃毒、OCR 移 threadpool、公開上傳 per-IP 限流</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="38" customHeight="1">
       <c r="A5" s="40" t="inlineStr">
@@ -877,6 +893,11 @@
           <t>HR 校準權重與公平性檢核</t>
         </is>
       </c>
+      <c r="E5" s="40" t="inlineStr">
+        <is>
+          <t>已上線並強化：技能同義詞＋模糊比對、門檻軟化（比例／鄰近城市／near_miss）、雙語職稱、媒合評估報表</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="38" customHeight="1">
       <c r="A6" s="41" t="inlineStr">
@@ -899,6 +920,11 @@
           <t>公司 Logo／色票／導覽／SSO 規格</t>
         </is>
       </c>
+      <c r="E6" s="41" t="inlineStr">
+        <is>
+          <t>角色化介面上線；佈署強化：nginx 安全標頭／CSP、容器非 root、API 綁 loopback、/health 實檢、pip-audit CI</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="42" t="inlineStr">
@@ -911,8 +937,6 @@
           <t>「已完成 MVP」供內部展示／試用；正式處理真實個資前仍需樣本校準、資安檢核與 UAT。</t>
         </is>
       </c>
-      <c r="C8" s="43" t="n"/>
-      <c r="D8" s="43" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A2:D6"/>
@@ -971,7 +995,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>啟動 2026-07-20 ｜ v1.2：2026-07-14 更新 ｜ 色塊＝工作期間，◆＝里程碑</t>
+          <t>啟動 2026-07-20 ｜ v1.3：2026-07-16 更新 ｜ 實際進度：Phase 1–5 已完成、Phase 6 部分、已完成 LAN 內網試用部署（遠早於原排程）；剩正式上線硬化 ｜ 色塊＝工作期間，◆＝里程碑</t>
         </is>
       </c>
     </row>
@@ -1653,13 +1677,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
     <col width="30" customWidth="1" min="3" max="3"/>
     <col width="34" customWidth="1" min="4" max="4"/>
+    <col width="48" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1683,6 +1708,11 @@
           <t>對 HR 的意義</t>
         </is>
       </c>
+      <c r="E1" s="3" t="inlineStr">
+        <is>
+          <t>實際狀態（2026-07-16）</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="9" t="inlineStr">
@@ -1705,6 +1735,11 @@
           <t>欄位與流程共識</t>
         </is>
       </c>
+      <c r="E2" s="8" t="inlineStr">
+        <is>
+          <t>已達</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="9" t="inlineStr">
@@ -1727,6 +1762,11 @@
           <t>可開始集中管理人才</t>
         </is>
       </c>
+      <c r="E3" s="8" t="inlineStr">
+        <is>
+          <t>已達（提前）</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="28" t="inlineStr">
@@ -1749,6 +1789,11 @@
           <t>建檔 15 分鐘 → 30 秒</t>
         </is>
       </c>
+      <c r="E4" s="29" t="inlineStr">
+        <is>
+          <t>已達（提前，內網試用）</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="9" t="inlineStr">
@@ -1771,6 +1816,11 @@
           <t>主管需求數位化</t>
         </is>
       </c>
+      <c r="E5" s="8" t="inlineStr">
+        <is>
+          <t>已達（提前）</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="9" t="inlineStr">
@@ -1793,6 +1843,11 @@
           <t>開缺 1 小時內拿到名單</t>
         </is>
       </c>
+      <c r="E6" s="8" t="inlineStr">
+        <is>
+          <t>已達（提前，且已強化＋評估報表）</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="9" t="inlineStr">
@@ -1813,6 +1868,11 @@
       <c r="D7" s="8" t="inlineStr">
         <is>
           <t>完整生態圈運作</t>
+        </is>
+      </c>
+      <c r="E7" s="8" t="inlineStr">
+        <is>
+          <t>功能大致齊備；尚缺正式上線硬化（HTTPS／備份還原／監控／MFA／真實資料 UAT）</t>
         </is>
       </c>
     </row>
@@ -1827,7 +1887,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:G9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -1836,6 +1896,7 @@
     <col width="50" customWidth="1" min="4" max="4"/>
     <col width="44" customWidth="1" min="5" max="5"/>
     <col width="9" customWidth="1" min="6" max="6"/>
+    <col width="44" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1869,6 +1930,11 @@
           <t>里程碑</t>
         </is>
       </c>
+      <c r="G1" s="3" t="inlineStr">
+        <is>
+          <t>完成度（2026-07-16）</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="42" customHeight="1">
       <c r="A2" s="30" t="inlineStr">
@@ -1901,6 +1967,11 @@
           <t>—</t>
         </is>
       </c>
+      <c r="G2" s="9" t="inlineStr">
+        <is>
+          <t>完成</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="42" customHeight="1">
       <c r="A3" s="31" t="inlineStr">
@@ -1933,6 +2004,11 @@
           <t>—</t>
         </is>
       </c>
+      <c r="G3" s="9" t="inlineStr">
+        <is>
+          <t>完成（含認證強化）</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="42" customHeight="1">
       <c r="A4" s="32" t="inlineStr">
@@ -1965,6 +2041,11 @@
           <t>M1</t>
         </is>
       </c>
+      <c r="G4" s="9" t="inlineStr">
+        <is>
+          <t>完成</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="42" customHeight="1">
       <c r="A5" s="33" t="inlineStr">
@@ -1997,6 +2078,11 @@
           <t>M2</t>
         </is>
       </c>
+      <c r="G5" s="9" t="inlineStr">
+        <is>
+          <t>大致完成（監控資料夾／效能承諾未做）</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="42" customHeight="1">
       <c r="A6" s="34" t="inlineStr">
@@ -2029,6 +2115,11 @@
           <t>M3</t>
         </is>
       </c>
+      <c r="G6" s="9" t="inlineStr">
+        <is>
+          <t>完成（Email 通知未做）</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="42" customHeight="1">
       <c r="A7" s="35" t="inlineStr">
@@ -2061,6 +2152,11 @@
           <t>M4</t>
         </is>
       </c>
+      <c r="G7" s="9" t="inlineStr">
+        <is>
+          <t>完成並強化（含準確率改進＋媒合評估報表）</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="42" customHeight="1">
       <c r="A8" s="36" t="inlineStr">
@@ -2093,6 +2189,11 @@
           <t>—</t>
         </is>
       </c>
+      <c r="G8" s="9" t="inlineStr">
+        <is>
+          <t>部分完成（報表與資安強化已完成大半；保存期限自動化／壓測／備份／TLS 未做）</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="42" customHeight="1">
       <c r="A9" s="37" t="inlineStr">
@@ -2123,6 +2224,11 @@
       <c r="F9" s="9" t="inlineStr">
         <is>
           <t>M5</t>
+        </is>
+      </c>
+      <c r="G9" s="9" t="inlineStr">
+        <is>
+          <t>部分（LAN 內網試用已完成；真實資料 UAT／HTTPS／備份還原 未做）</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: harden consent privacy and release tracking
</commit_message>
<xml_diff>
--- a/docs/TalentHub_專案時程表.xlsx
+++ b/docs/TalentHub_專案時程表.xlsx
@@ -787,7 +787,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="38" t="inlineStr">
         <is>
-          <t>TalentHub 平行工作流進度（更新至 2026-07-16）</t>
+          <t>TalentHub 平行工作流進度（更新至 2026-08-04）</t>
         </is>
       </c>
     </row>
@@ -814,118 +814,119 @@
       </c>
       <c r="E2" s="39" t="inlineStr">
         <is>
-          <t>現況（2026-07-16）</t>
+          <t>現況（2026-08-04）</t>
         </is>
       </c>
     </row>
     <row r="3" ht="38" customHeight="1">
       <c r="A3" s="40" t="inlineStr">
         <is>
-          <t>多角色權限與資料範圍</t>
+          <t>角色權限、面試與 IT 後台</t>
         </is>
       </c>
       <c r="B3" s="40" t="inlineStr">
         <is>
-          <t>已完成 MVP</t>
+          <t>強化完成／本機驗證通過</t>
         </is>
       </c>
       <c r="C3" s="40" t="inlineStr">
         <is>
-          <t>IT／HR／主管依角色與資料範圍操作</t>
+          <t>角色範圍面試題、逐題重產、部門資料隔離、IT 後台邊界</t>
         </is>
       </c>
       <c r="D3" s="40" t="inlineStr">
         <is>
-          <t>三角色 UAT 與越權測試</t>
+          <t>三角色越權 UAT；驗證主管僅看遮罩資料且不可下載原始履歷</t>
         </is>
       </c>
       <c r="E3" s="40" t="inlineStr">
         <is>
-          <t>已上線；認證強化：帳號級自動過期鎖定、強制首登改密、密碼重設令 token 失效、refresh 重用偵測</t>
+          <t>角色題組、逐題重產、同意撤回、後端登出與權限 hardening 已完成；本機驗證通過，待 PR／UAT</t>
         </is>
       </c>
     </row>
     <row r="4" ht="38" customHeight="1">
       <c r="A4" s="41" t="inlineStr">
         <is>
-          <t>104／1111 OCR 固定欄位入庫</t>
+          <t>人才入庫、搜尋與去識別化</t>
         </is>
       </c>
       <c r="B4" s="41" t="inlineStr">
         <is>
-          <t>已完成 MVP</t>
+          <t>已完成 MVP／待 UAT</t>
         </is>
       </c>
       <c r="C4" s="41" t="inlineStr">
         <is>
-          <t>來源模板、固定欄位、信心分數、校對後入庫</t>
+          <t>整合人才入庫、OCR／解析／去重、候選搜尋、安全履歷</t>
         </is>
       </c>
       <c r="D4" s="41" t="inlineStr">
         <is>
-          <t>各 10 份授權去識別樣本校準</t>
+          <t>授權真實版型驗收；保存期限與撤回後處置定案</t>
         </is>
       </c>
       <c r="E4" s="41" t="inlineStr">
         <is>
-          <t>解析／OCR／去重／並排校對已上線；上傳安全：非 dev fail-closed 掃毒、OCR 移 threadpool、公開上傳 per-IP 限流</t>
+          <t>入庫、搜尋、去識別化及法遵檢查已完成；掃描 PDF／OCR、多版型仍需 UAT</t>
         </is>
       </c>
     </row>
     <row r="5" ht="38" customHeight="1">
       <c r="A5" s="40" t="inlineStr">
         <is>
-          <t>可解釋人才職缺配對</t>
+          <t>媒合、法遵與 AI 輔助</t>
         </is>
       </c>
       <c r="B5" s="40" t="inlineStr">
         <is>
-          <t>已完成 MVP</t>
+          <t>已完成 MVP／待校準</t>
         </is>
       </c>
       <c r="C5" s="40" t="inlineStr">
         <is>
-          <t>必要條件與多面向分數、排序原因</t>
+          <t>六面向可解釋媒合、JD／面試題法遵檢查、Gemini 備援</t>
         </is>
       </c>
       <c r="D5" s="40" t="inlineStr">
         <is>
-          <t>HR 校準權重與公平性檢核</t>
+          <t>HR 校準／公平性檢核；核准 AI 與最小傳送欄位</t>
         </is>
       </c>
       <c r="E5" s="40" t="inlineStr">
         <is>
-          <t>已上線並強化：技能同義詞＋模糊比對、門檻軟化（比例／鄰近城市／near_miss）、雙語職稱、媒合評估報表</t>
+          <t>媒合與不當內容檢查已完成；AI 不參與錄取，雲端使用與傳送欄位待政策核准</t>
         </is>
       </c>
     </row>
     <row r="6" ht="38" customHeight="1">
       <c r="A6" s="41" t="inlineStr">
         <is>
-          <t>角色化互動介面／官網整合</t>
+          <t>公開網站、UAT 與主線部署</t>
         </is>
       </c>
       <c r="B6" s="41" t="inlineStr">
         <is>
-          <t>已完成介面基線</t>
+          <t>本機驗證通過／待 PR、UAT</t>
         </is>
       </c>
       <c r="C6" s="41" t="inlineStr">
         <is>
-          <t>角色導覽、任務提示、響應式工作台</t>
+          <t>TalentHub 公開入口、同意版本、完整測試、PR／IT 部署檢核</t>
         </is>
       </c>
       <c r="D6" s="41" t="inlineStr">
         <is>
-          <t>公司 Logo／色票／導覽／SSO 規格</t>
+          <t>法務啟用首版同意書；公開職缺策略；HTTPS、備份還原、監控、MFA</t>
         </is>
       </c>
       <c r="E6" s="41" t="inlineStr">
         <is>
-          <t>角色化介面上線；佈署強化：nginx 安全標頭／CSP、容器非 root、API 綁 loopback、/health 實檢、pip-audit CI</t>
-        </is>
-      </c>
-    </row>
+          <t>公開入口與資安 hardening 已完成本機驗證；待 PR 合併 main、內網 UAT，再由 IT 部署</t>
+        </is>
+      </c>
+    </row>
+    <row r="7"/>
     <row r="8">
       <c r="A8" s="42" t="inlineStr">
         <is>
@@ -934,7 +935,7 @@
       </c>
       <c r="B8" s="43" t="inlineStr">
         <is>
-          <t>「已完成 MVP」供內部展示／試用；正式處理真實個資前仍需樣本校準、資安檢核與 UAT。</t>
+          <t>本機整合驗證已通過（後端 261 項測試、HR 後台與公開前端正式建置）；尚需 PR 審查、UAT 及 IT 上線關卡，不能視為已正式發布。</t>
         </is>
       </c>
     </row>
@@ -988,14 +989,14 @@
     <row r="1" ht="26" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>TalentHub 專案時程甘特圖</t>
+          <t>TalentHub 專案時程甘特圖（更新至 2026-08-04）</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>啟動 2026-07-20 ｜ v1.3：2026-07-16 更新 ｜ 實際進度：Phase 1–5 已完成、Phase 6 部分、已完成 LAN 內網試用部署（遠早於原排程）；剩正式上線硬化 ｜ 色塊＝工作期間，◆＝里程碑</t>
+          <t>啟動 2026-07-20 ｜ v1.4：2026-08-04 更新 ｜ 實際進度：P0–P5 功能大致完成、P6 hardening 本機整合驗證通過（後端 261 項、兩個前端 build）；下一關＝PR 審查、完整 UAT、合併 main、IT 部署檢核 ｜ 色塊＝基準排程，◆＝里程碑</t>
         </is>
       </c>
     </row>
@@ -1187,7 +1188,7 @@
       </c>
       <c r="B5" s="8" t="inlineStr">
         <is>
-          <t>欄位定稿、104/1111 履歷樣本蒐集、環境與 SMTP 盤點、KPI 基準量測</t>
+          <t>政策／欄位定稿、角色與資料範圍、104／1111 授權樣本、KPI 基準</t>
         </is>
       </c>
       <c r="C5" s="9" t="inlineStr">
@@ -1239,7 +1240,7 @@
       </c>
       <c r="B6" s="8" t="inlineStr">
         <is>
-          <t>Repo/CI、Docker Compose、Alembic 建表、登入/JWT/RBAC、使用者與部門</t>
+          <t>Repo／CI、Docker、Migration、JWT／RBAC、部門隔離、IT 後台與登出 hardening</t>
         </is>
       </c>
       <c r="C6" s="9" t="inlineStr">
@@ -1291,7 +1292,7 @@
       </c>
       <c r="B7" s="8" t="inlineStr">
         <is>
-          <t>人才 CRUD＋子表、複合搜尋(pg_trgm)、標籤、狀態機、聯繫紀錄、技能字典</t>
+          <t>整合人才入庫、人才 CRUD、候選搜尋、標籤／狀態、聯繫紀錄與技能字典</t>
         </is>
       </c>
       <c r="C7" s="9" t="inlineStr">
@@ -1343,7 +1344,7 @@
       </c>
       <c r="B8" s="8" t="inlineStr">
         <is>
-          <t>Parser104/1111/Generic、批次上傳、校對介面、去重、監控資料夾、回歸測試</t>
+          <t>104／1111／Generic Parser、OCR、批次上傳、去重、校對、去識別化與回歸測試</t>
         </is>
       </c>
       <c r="C8" s="9" t="inlineStr">
@@ -1395,7 +1396,7 @@
       </c>
       <c r="B9" s="8" t="inlineStr">
         <is>
-          <t>需求單精靈、簽核流、職缺看板、站內＋Email 通知</t>
+          <t>需求單／簽核／職缺看板、JD 法遵檢查、站內通知（Email 待整合）</t>
         </is>
       </c>
       <c r="C9" s="9" t="inlineStr">
@@ -1447,7 +1448,7 @@
       </c>
       <c r="B10" s="8" t="inlineStr">
         <is>
-          <t>硬條件過濾＋六面向計分、推薦名單、配對工作台、主管回饋、遮罩</t>
+          <t>六面向可解釋媒合、角色範圍面試題、逐題重產、版本與主管回饋</t>
         </is>
       </c>
       <c r="C10" s="9" t="inlineStr">
@@ -1499,7 +1500,7 @@
       </c>
       <c r="B11" s="8" t="inlineStr">
         <is>
-          <t>四張報表、通知完善、保存期限排程與匿名化、資安強化、10 萬筆壓測</t>
+          <t>同意版本／撤回、保存期限、權限與資安 hardening、報表、壓測、備份／監控</t>
         </is>
       </c>
       <c r="C11" s="9" t="inlineStr">
@@ -1551,7 +1552,7 @@
       </c>
       <c r="B12" s="8" t="inlineStr">
         <is>
-          <t>UAT、歷史履歷回灌、教育訓練、正式上線、備份還原演練</t>
+          <t>完整 UAT／CI／E2E、PR 合併 main、教育訓練、HTTPS、備份還原與 IT 部署</t>
         </is>
       </c>
       <c r="C12" s="9" t="inlineStr">
@@ -1710,7 +1711,7 @@
       </c>
       <c r="E1" s="3" t="inlineStr">
         <is>
-          <t>實際狀態（2026-07-16）</t>
+          <t>實際狀態（2026-08-04）</t>
         </is>
       </c>
     </row>
@@ -1737,7 +1738,7 @@
       </c>
       <c r="E2" s="8" t="inlineStr">
         <is>
-          <t>已達</t>
+          <t>已達（需求與基礎政策已盤點）</t>
         </is>
       </c>
     </row>
@@ -1764,7 +1765,7 @@
       </c>
       <c r="E3" s="8" t="inlineStr">
         <is>
-          <t>已達（提前）</t>
+          <t>已達（提前：整合人才入庫、候選搜尋與角色資料範圍）</t>
         </is>
       </c>
     </row>
@@ -1786,12 +1787,12 @@
       </c>
       <c r="D4" s="29" t="inlineStr">
         <is>
-          <t>建檔 15 分鐘 → 30 秒</t>
+          <t>縮短結構化建檔時間（待 UAT 量測）</t>
         </is>
       </c>
       <c r="E4" s="29" t="inlineStr">
         <is>
-          <t>已達（提前，內網試用）</t>
+          <t>已達（提前：解析／OCR／去重／去識別化；真實版型待 UAT）</t>
         </is>
       </c>
     </row>
@@ -1818,7 +1819,7 @@
       </c>
       <c r="E5" s="8" t="inlineStr">
         <is>
-          <t>已達（提前）</t>
+          <t>已達（提前：職缺流程與法遵檢查；Email 通知待整合）</t>
         </is>
       </c>
     </row>
@@ -1835,17 +1836,17 @@
       </c>
       <c r="C6" s="8" t="inlineStr">
         <is>
-          <t>智慧配對上線</t>
+          <t>智慧配對與角色化面試上線</t>
         </is>
       </c>
       <c r="D6" s="8" t="inlineStr">
         <is>
-          <t>開缺 1 小時內拿到名單</t>
+          <t>可解釋名單＋可控面試題流程</t>
         </is>
       </c>
       <c r="E6" s="8" t="inlineStr">
         <is>
-          <t>已達（提前，且已強化＋評估報表）</t>
+          <t>已達（提前：可解釋媒合、角色題組與逐題重產；待校準）</t>
         </is>
       </c>
     </row>
@@ -1872,7 +1873,7 @@
       </c>
       <c r="E7" s="8" t="inlineStr">
         <is>
-          <t>功能大致齊備；尚缺正式上線硬化（HTTPS／備份還原／監控／MFA／真實資料 UAT）</t>
+          <t>UAT 準備中：hardening 本機驗證通過；尚待 PR／UAT／HTTPS／備份還原／監控／MFA</t>
         </is>
       </c>
     </row>
@@ -1932,7 +1933,7 @@
       </c>
       <c r="G1" s="3" t="inlineStr">
         <is>
-          <t>完成度（2026-07-16）</t>
+          <t>完成度（2026-08-04）</t>
         </is>
       </c>
     </row>
@@ -1954,12 +1955,12 @@
       </c>
       <c r="D2" s="8" t="inlineStr">
         <is>
-          <t>欄位定稿、104/1111 履歷樣本蒐集、環境與 SMTP 盤點、KPI 基準量測</t>
+          <t>欄位／角色／資料範圍定稿、授權樣本、環境／SMTP／AI／KPI 盤點</t>
         </is>
       </c>
       <c r="E2" s="8" t="inlineStr">
         <is>
-          <t>欄位清單定稿、去識別化樣本庫、部署決策紀錄</t>
+          <t>欄位與政策清單、去識別化樣本庫、部署決策紀錄</t>
         </is>
       </c>
       <c r="F2" s="9" t="inlineStr">
@@ -1969,7 +1970,7 @@
       </c>
       <c r="G2" s="9" t="inlineStr">
         <is>
-          <t>完成</t>
+          <t>完成；程式品牌已統一 TalentHub；正式商標／網域、保存期限與 AI 核准待定</t>
         </is>
       </c>
     </row>
@@ -1991,12 +1992,12 @@
       </c>
       <c r="D3" s="8" t="inlineStr">
         <is>
-          <t>Repo/CI、Docker Compose、Alembic 建表、登入/JWT/RBAC、使用者與部門</t>
+          <t>Repo／CI、Docker、Migration、JWT／RBAC、使用者／部門、IT 後台、登出與權限 hardening</t>
         </is>
       </c>
       <c r="E3" s="8" t="inlineStr">
         <is>
-          <t>三種角色可登入且權限選單正確；一鍵起環境</t>
+          <t>三角色登入／導覽／範圍正確；refresh 撤銷；IT 不讀招募資料</t>
         </is>
       </c>
       <c r="F3" s="9" t="inlineStr">
@@ -2006,7 +2007,7 @@
       </c>
       <c r="G3" s="9" t="inlineStr">
         <is>
-          <t>完成（含認證強化）</t>
+          <t>核心完成；hardening 本機整合驗證通過，待 PR／UAT</t>
         </is>
       </c>
     </row>
@@ -2028,12 +2029,12 @@
       </c>
       <c r="D4" s="8" t="inlineStr">
         <is>
-          <t>人才 CRUD＋子表、複合搜尋(pg_trgm)、標籤、狀態機、聯繫紀錄、技能字典</t>
+          <t>整合人才入庫、人才 CRUD、候選搜尋、標籤／狀態、聯繫紀錄、技能字典</t>
         </is>
       </c>
       <c r="E4" s="8" t="inlineStr">
         <is>
-          <t>手動建檔並以技能+年資+地區 2 秒搜得；聯繫紀錄可追蹤</t>
+          <t>可建檔入庫並以技能＋年資＋地區 2 秒搜得；部門資料範圍正確</t>
         </is>
       </c>
       <c r="F4" s="9" t="inlineStr">
@@ -2043,7 +2044,7 @@
       </c>
       <c r="G4" s="9" t="inlineStr">
         <is>
-          <t>完成</t>
+          <t>完成；真實資料量與越權情境待 UAT</t>
         </is>
       </c>
     </row>
@@ -2065,12 +2066,12 @@
       </c>
       <c r="D5" s="8" t="inlineStr">
         <is>
-          <t>Parser104/1111/Generic、批次上傳、校對介面、去重、監控資料夾、回歸測試</t>
+          <t>104／1111／Generic Parser、OCR、批次上傳、校對、去重、去識別化與回歸測試</t>
         </is>
       </c>
       <c r="E5" s="8" t="inlineStr">
         <is>
-          <t>30 份 104 履歷 3 分鐘解析、自動入庫率≥70%、重複自動標示→試營運</t>
+          <t>授權樣本可解析／標示重複；原始／安全版本分離，核准後使用</t>
         </is>
       </c>
       <c r="F5" s="9" t="inlineStr">
@@ -2080,7 +2081,7 @@
       </c>
       <c r="G5" s="9" t="inlineStr">
         <is>
-          <t>大致完成（監控資料夾／效能承諾未做）</t>
+          <t>大致完成；掃描 PDF／OCR／多版型與監控資料夾待 UAT／後續</t>
         </is>
       </c>
     </row>
@@ -2102,12 +2103,12 @@
       </c>
       <c r="D6" s="8" t="inlineStr">
         <is>
-          <t>需求單精靈、簽核流、職缺看板、站內＋Email 通知</t>
+          <t>需求單簽核、職缺看板、JD 法遵檢查、站內／Email 通知</t>
         </is>
       </c>
       <c r="E6" s="8" t="inlineStr">
         <is>
-          <t>主管 5 分鐘完成需求單；HR 即刻收到通知並可核准</t>
+          <t>主管可送審、HR 可核准；不當條件有警示；狀態可追蹤</t>
         </is>
       </c>
       <c r="F6" s="9" t="inlineStr">
@@ -2117,7 +2118,7 @@
       </c>
       <c r="G6" s="9" t="inlineStr">
         <is>
-          <t>完成（Email 通知未做）</t>
+          <t>核心完成（含 JD 法遵）；Email 通知／公開職缺策略待定</t>
         </is>
       </c>
     </row>
@@ -2139,12 +2140,12 @@
       </c>
       <c r="D7" s="8" t="inlineStr">
         <is>
-          <t>硬條件過濾＋六面向計分、推薦名單、配對工作台、主管回饋、遮罩</t>
+          <t>必要條件＋六面向媒合、near miss、角色範圍面試題、逐題重產與回饋</t>
         </is>
       </c>
       <c r="E7" s="8" t="inlineStr">
         <is>
-          <t>核准 1 分鐘產出 Top20 附原因；回饋即時回寫；抽查認可≥80%</t>
+          <t>Top20 附原因；角色題組正確；重產不影響其他題與歷史；法遵通過</t>
         </is>
       </c>
       <c r="F7" s="9" t="inlineStr">
@@ -2154,7 +2155,7 @@
       </c>
       <c r="G7" s="9" t="inlineStr">
         <is>
-          <t>完成並強化（含準確率改進＋媒合評估報表）</t>
+          <t>完成並強化；本機驗證通過，媒合效果待 UAT 校準</t>
         </is>
       </c>
     </row>
@@ -2176,12 +2177,12 @@
       </c>
       <c r="D8" s="8" t="inlineStr">
         <is>
-          <t>四張報表、通知完善、保存期限排程與匿名化、資安強化、10 萬筆壓測</t>
+          <t>報表、同意版本／撤回、保存期限、登出撤銷、權限／資安 hardening、壓測</t>
         </is>
       </c>
       <c r="E8" s="8" t="inlineStr">
         <is>
-          <t>docs/02 非功能需求全數達標</t>
+          <t>撤回即停止利用；資料最小化；越權阻擋；備份／監控／TLS 檢核可追蹤</t>
         </is>
       </c>
       <c r="F8" s="9" t="inlineStr">
@@ -2191,7 +2192,7 @@
       </c>
       <c r="G8" s="9" t="inlineStr">
         <is>
-          <t>部分完成（報表與資安強化已完成大半；保存期限自動化／壓測／備份／TLS 未做）</t>
+          <t>進行中：法遵／權限／資安 hardening 本機驗證通過；首版同意書、保存排程、TLS／備份／監控／MFA 待法務或 IT</t>
         </is>
       </c>
     </row>
@@ -2213,12 +2214,12 @@
       </c>
       <c r="D9" s="8" t="inlineStr">
         <is>
-          <t>UAT、歷史履歷回灌、教育訓練、正式上線、備份還原演練</t>
+          <t>完整 UAT、歷史履歷回灌、PR 合併 main、教育訓練、正式發布與回滾演練</t>
         </is>
       </c>
       <c r="E9" s="8" t="inlineStr">
         <is>
-          <t>正式環境上線、備份還原演練通過、KPI 儀表板啟用</t>
+          <t>完整 CI／E2E／UAT 通過；主線版本可部署；HTTPS／備份還原／監控／回滾有證據</t>
         </is>
       </c>
       <c r="F9" s="9" t="inlineStr">
@@ -2228,7 +2229,7 @@
       </c>
       <c r="G9" s="9" t="inlineStr">
         <is>
-          <t>部分（LAN 內網試用已完成；真實資料 UAT／HTTPS／備份還原 未做）</t>
+          <t>待執行：本機 261 項測試與兩個前端建置已通過；下一關為 PR 審查／UAT／IT 部署驗證</t>
         </is>
       </c>
     </row>

</xml_diff>